<commit_message>
Sync TEST_STUB_SERVICE_BASE_URL callback templating in BEFTA master and generated JSON
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/GenericDefinitionFile.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/GenericDefinitionFile.xlsx
@@ -1799,7 +1799,7 @@
     <t>Create a case</t>
   </si>
   <si>
-    <t>http://ccd-test-stubs-service-aat.service.core-compute-aat.internal/case_type/fe-functional-test/mid_event_dynamic_list</t>
+    <t>${TEST_STUB_SERVICE_BASE_URL:http://ccd-test-stubs-service-aat.service.core-compute-aat.internal}/case_type/fe-functional-test/mid_event_dynamic_list</t>
   </si>
   <si>
     <t>Y</t>
@@ -2443,7 +2443,7 @@
     <t>Trigger callback warnings</t>
   </si>
   <si>
-    <t>http://ccd-test-stubs-service-aat.service.core-compute-aat.internal/callback_returning_warnings</t>
+    <t>${TEST_STUB_SERVICE_BASE_URL:http://ccd-test-stubs-service-aat.service.core-compute-aat.internal}/callback_returning_warnings</t>
   </si>
   <si>
     <t>triggerCallbackErrorsAndWarnings</t>
@@ -2455,7 +2455,7 @@
     <t>Trigger callback errors and warnings</t>
   </si>
   <si>
-    <t>http://ccd-test-stubs-service-aat.service.core-compute-aat.internal/callback_returning_errors_and_warnings</t>
+    <t>${TEST_STUB_SERVICE_BASE_URL:http://ccd-test-stubs-service-aat.service.core-compute-aat.internal}/callback_returning_errors_and_warnings</t>
   </si>
   <si>
     <t>test@gmail.com</t>

</xml_diff>